<commit_message>
feat(Q4): P0 三审修正 — chance constraint + 过渡时间 + 双解对照
按 Q4_三审综合 P0 执行:
1. chance constraint (z=1.645 = 90% 单侧): d - z·σ_d ≥ d_min, d + z·σ_d
   ≤ d_max, v + z·σ_v ≤ v_max, σ_v = 5%·|v|
2. ILP 时段约束加 ε = 0.1s 过渡时间 (武器/相机切换)
3. main 改双解对照: 标称 vs 鲁棒, 输出公共/仅标称/仅鲁棒
4. JSON summary 加目标函数语义说明 (完成数 = 不同目标数)

意外发现 (vs Claude 预测 17-18 任务):
- 标称解 20 任务 (8 射击 + 12 拍照, 期望命中 6.80)
- 鲁棒解 21 任务 (9 射击 + 12 拍照, 期望命中 7.65)
- ILP 全局重组让 S06 从 462.2 d=5.02 (边界) 移到 460.5 d=6.07 (安全)
- 同时新增 S05/S01/P15/P17 等候选, 替代 S13/P10 等边界候选
- σ_d ≈ 0.6 m, 鲁棒下界 d ≥ 5.99 / d ≤ 39.01

主交付切换为鲁棒解 21 任务. 标称解保留在 JSON 中作对照.
result_filled.xlsx 已用鲁棒解填充.
</commit_message>
<xml_diff>
--- a/xk/output/Q4_result_filled.xlsx
+++ b/xk/output/Q4_result_filled.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="15.77734375" customWidth="1" min="4" max="4"/>
@@ -646,10 +646,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>460.7</v>
+        <v>459</v>
       </c>
       <c r="E7" t="n">
-        <v>462.2</v>
+        <v>460.5</v>
       </c>
     </row>
     <row r="8">
@@ -658,7 +658,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>463.2</v>
+        <v>461.7</v>
       </c>
       <c r="E8" t="n">
-        <v>463.7</v>
+        <v>462.2</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +679,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -688,10 +688,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>466.8</v>
+        <v>463.2</v>
       </c>
       <c r="E9" t="n">
-        <v>467.3</v>
+        <v>463.7</v>
       </c>
     </row>
     <row r="10">
@@ -700,19 +700,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>S03</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>468.1</v>
+        <v>464.9</v>
       </c>
       <c r="E10" t="n">
-        <v>469.6</v>
+        <v>465.4</v>
       </c>
     </row>
     <row r="11">
@@ -721,19 +721,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>477</v>
+        <v>466.8</v>
       </c>
       <c r="E11" t="n">
-        <v>478.5</v>
+        <v>467.3</v>
       </c>
     </row>
     <row r="12">
@@ -742,19 +742,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>S04</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>479.4</v>
+        <v>467.8</v>
       </c>
       <c r="E12" t="n">
-        <v>479.9</v>
+        <v>469.3</v>
       </c>
     </row>
     <row r="13">
@@ -763,19 +763,19 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>480.6</v>
+        <v>477.3</v>
       </c>
       <c r="E13" t="n">
-        <v>481.1</v>
+        <v>478.8</v>
       </c>
     </row>
     <row r="14">
@@ -784,19 +784,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>S03</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>492.9</v>
+        <v>479.1</v>
       </c>
       <c r="E14" t="n">
-        <v>493.4</v>
+        <v>480.6</v>
       </c>
     </row>
     <row r="15">
@@ -805,19 +805,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>494.3</v>
+        <v>480.7</v>
       </c>
       <c r="E15" t="n">
-        <v>494.8</v>
+        <v>482.2</v>
       </c>
     </row>
     <row r="16">
@@ -826,7 +826,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -835,10 +835,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>507.8</v>
+        <v>493.2</v>
       </c>
       <c r="E16" t="n">
-        <v>508.3</v>
+        <v>493.7</v>
       </c>
     </row>
     <row r="17">
@@ -847,19 +847,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>511.2</v>
+        <v>493.8</v>
       </c>
       <c r="E17" t="n">
-        <v>512.7</v>
+        <v>494.3</v>
       </c>
     </row>
     <row r="18">
@@ -868,19 +868,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>P01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>516.7</v>
+        <v>508.1</v>
       </c>
       <c r="E18" t="n">
-        <v>518.2</v>
+        <v>508.6</v>
       </c>
     </row>
     <row r="19">
@@ -889,7 +889,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>650.3</v>
+        <v>511.2</v>
       </c>
       <c r="E19" t="n">
-        <v>651.8</v>
+        <v>512.7</v>
       </c>
     </row>
     <row r="20">
@@ -910,7 +910,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>S14</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>750.1</v>
+        <v>516.7</v>
       </c>
       <c r="E20" t="n">
-        <v>751.6</v>
+        <v>518.2</v>
       </c>
     </row>
     <row r="21">
@@ -931,7 +931,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>S15</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -940,13 +940,34 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>762.3</v>
+        <v>749.2</v>
       </c>
       <c r="E21" t="n">
-        <v>763.8</v>
-      </c>
-    </row>
-    <row r="22"/>
+        <v>750.7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>766.2</v>
+      </c>
+      <c r="E22" t="n">
+        <v>767.7</v>
+      </c>
+    </row>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>